<commit_message>
Build final Head lamp Excel with cross-row AI Review findings merged in
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions_gpt5.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions_gpt5.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -3242,7 +3242,11 @@
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
-      <c r="AX20" s="223" t="inlineStr"/>
+      <c r="AX20" s="223" t="inlineStr">
+        <is>
+          <t>Compare to IMPROPER LOCKING / POOR LOCKING (rows 22-23): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
       <c r="AY20" s="223" t="inlineStr"/>
     </row>
     <row r="21" ht="153" customFormat="1" customHeight="1" s="8">
@@ -3884,7 +3888,7 @@
       </c>
       <c r="AX26" s="223" t="inlineStr">
         <is>
-          <t>Plant listed only cosmetic/NVH End User effects for this row (lens crack, LED burnout, water ingress, rattling, discomfort) - no beam-alignment/visibility/accident-risk option, unlike the near-identical 'Prefit bolts' step (same mounting joint) which lists those and scored S=10. If loose/missing screws can also misalign the beam, add that effect to this row's own Effect cell in the plant's source Excel so AI severity reflects it; do not change AI/prompt logic to compensate - broadening the effect list plant-wide risks re-inflating severity on unrelated rows (a documented past failure mode of this pipeline).</t>
+          <t>Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
         </is>
       </c>
       <c r="AY26" s="223" t="inlineStr"/>
@@ -4050,7 +4054,11 @@
           <t>- Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED - OVER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
-      <c r="AX28" s="223" t="inlineStr"/>
+      <c r="AX28" s="223" t="inlineStr">
+        <is>
+          <t>Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
       <c r="AY28" s="223" t="inlineStr"/>
     </row>
     <row r="29" ht="165" customFormat="1" customHeight="1" s="13">
@@ -4143,7 +4151,11 @@
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: TORQUE NOT ACHIEVED-UNDER TORQUE. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
-      <c r="AX29" s="223" t="inlineStr"/>
+      <c r="AX29" s="223" t="inlineStr">
+        <is>
+          <t>Compare to OPERATOR FAILED TO PREFIT BOLTS (rows 24-25): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
+        </is>
+      </c>
       <c r="AY29" s="223" t="inlineStr"/>
     </row>
     <row r="30" customFormat="1" s="18"/>

</xml_diff>

<commit_message>
Fix false-positive cross-row flag: require matching Cause mechanism
Manual review found step5c flagged 'Fitment not firm/wrong selection'
against 'Improper locking' - different physical mechanisms (wrong part
installed vs. connector not locked), just because both touch beam
alignment in the abstract. Removed that entry from the current output
and tightened the prompt to require the two rows' actual Failure Cause
text describe the same physical action, not just a vaguely related
topic - now shown directly in the prompt so the LLM can check it
itself instead of inferring from Failure Mode wording alone.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MG2nzeeWa5SnWqcTDjXsda
</commit_message>
<xml_diff>
--- a/pfmea_ai/NEW_PFMEA__with_suggestions_gpt5.xlsx
+++ b/pfmea_ai/NEW_PFMEA__with_suggestions_gpt5.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Head lamp" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Grill fitment-High" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Grill fitment-Low" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Side seal" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -3242,11 +3242,7 @@
 - Same Failure Cause text is also used, verbatim, on a different Failure Mode: SCRATCH / DAMAGE ON HEAD LAMP. Verify this Cause actually belongs to this row and wasn't copy-pasted.</t>
         </is>
       </c>
-      <c r="AX20" s="223" t="inlineStr">
-        <is>
-          <t>Compare to IMPROPER LOCKING / POOR LOCKING (rows 22-23): missing incorrect beam alignment, reduced road visibility, and accident-risk effects — review/add to this row's Effect cell if applicable.</t>
-        </is>
-      </c>
+      <c r="AX20" s="223" t="inlineStr"/>
       <c r="AY20" s="223" t="inlineStr"/>
     </row>
     <row r="21" ht="153" customFormat="1" customHeight="1" s="8">

</xml_diff>